<commit_message>
Fix: Changed Cars Insurance to CORS (wife's CC consolidation)
Co-authored-by: jbox662 <jbox662@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Family_Budget.xlsx
+++ b/Family_Budget.xlsx
@@ -63,9 +63,6 @@
     <t>Car Payment</t>
   </si>
   <si>
-    <t>Cars Insurance</t>
-  </si>
-  <si>
     <t>Boat</t>
   </si>
   <si>
@@ -133,6 +130,9 @@
   </si>
   <si>
     <t>Credit Card Consolidation</t>
+  </si>
+  <si>
+    <t>CORS (Wife CC Consolidation)</t>
   </si>
   <si>
     <t>Debt Total</t>
@@ -1466,7 +1466,7 @@
         <v>49</v>
       </c>
       <c r="E6" s="8">
-        <f>B21</f>
+        <f>B20</f>
         <v>0</v>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
         <v>50</v>
       </c>
       <c r="E7" s="8">
-        <f>B28</f>
+        <f>B27</f>
         <v>0</v>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
         <v>51</v>
       </c>
       <c r="E8" s="8">
-        <f>B37</f>
+        <f>B36</f>
         <v>0</v>
       </c>
     </row>
@@ -1506,7 +1506,7 @@
         <v>52</v>
       </c>
       <c r="E9" s="8">
-        <f>B43</f>
+        <f>B42</f>
         <v>0</v>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="6">
-        <v>519</v>
+        <v>565</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -1589,38 +1589,38 @@
         <v>16</v>
       </c>
       <c r="B19" s="6">
-        <v>565</v>
+        <v>800</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="6">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="9" t="s">
+      <c r="B20" s="10">
+        <f>SUM(B16:B19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="10">
-        <f>SUM(B16:B20)</f>
-        <v>0</v>
-      </c>
+      <c r="B22" s="3"/>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="3"/>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>4</v>
+      <c r="B24" s="6">
+        <v>641</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -1628,7 +1628,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="6">
-        <v>641</v>
+        <v>362.9</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -1636,38 +1636,38 @@
         <v>21</v>
       </c>
       <c r="B26" s="6">
-        <v>362.9</v>
+        <v>300</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="6">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
-      <c r="A28" s="9" t="s">
+      <c r="B27" s="10">
+        <f>SUM(B24:B26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="10">
-        <f>SUM(B25:B27)</f>
-        <v>0</v>
-      </c>
+      <c r="B29" s="3"/>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B30" s="3"/>
-    </row>
-    <row r="31" spans="1:2">
-      <c r="A31" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>4</v>
+      <c r="B31" s="6">
+        <v>400</v>
       </c>
     </row>
     <row r="32" spans="1:2">
@@ -1675,7 +1675,7 @@
         <v>25</v>
       </c>
       <c r="B32" s="6">
-        <v>400</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:2">
@@ -1683,7 +1683,7 @@
         <v>26</v>
       </c>
       <c r="B33" s="6">
-        <v>85</v>
+        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -1691,7 +1691,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="6">
-        <v>120</v>
+        <v>550</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -1699,38 +1699,38 @@
         <v>28</v>
       </c>
       <c r="B35" s="6">
-        <v>550</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B36" s="6">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2">
-      <c r="A37" s="9" t="s">
+      <c r="B36" s="10">
+        <f>SUM(B31:B35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B37" s="10">
-        <f>SUM(B32:B36)</f>
-        <v>0</v>
-      </c>
+      <c r="B38" s="3"/>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B39" s="3"/>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>4</v>
+      <c r="B40" s="6">
+        <v>104.17</v>
       </c>
     </row>
     <row r="41" spans="1:2">
@@ -1738,38 +1738,38 @@
         <v>32</v>
       </c>
       <c r="B41" s="6">
-        <v>104.17</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B42" s="6">
-        <v>34.3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2">
-      <c r="A43" s="9" t="s">
+      <c r="B42" s="10">
+        <f>SUM(B40:B41)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B43" s="10">
-        <f>SUM(B41:B42)</f>
-        <v>0</v>
-      </c>
+      <c r="B44" s="3"/>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B45" s="3"/>
-    </row>
-    <row r="46" spans="1:2">
-      <c r="A46" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>4</v>
+      <c r="B46" s="6">
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:2">
@@ -1777,7 +1777,7 @@
         <v>36</v>
       </c>
       <c r="B47" s="6">
-        <v>105</v>
+        <v>106.16</v>
       </c>
     </row>
     <row r="48" spans="1:2">
@@ -1785,7 +1785,7 @@
         <v>37</v>
       </c>
       <c r="B48" s="6">
-        <v>106.16</v>
+        <v>338</v>
       </c>
     </row>
     <row r="49" spans="1:2">
@@ -1793,7 +1793,7 @@
         <v>38</v>
       </c>
       <c r="B49" s="6">
-        <v>338</v>
+        <v>519</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -1801,7 +1801,7 @@
         <v>39</v>
       </c>
       <c r="B50" s="10">
-        <f>SUM(B47:B49)</f>
+        <f>SUM(B46:B49)</f>
         <v>0</v>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
         <v>46</v>
       </c>
       <c r="B60" s="10">
-        <f>B21+B28+B37+B43+B50+B57</f>
+        <f>B20+B27+B36+B42+B50+B57</f>
         <v>0</v>
       </c>
     </row>
@@ -1873,10 +1873,10 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A44:B44"/>
     <mergeCell ref="A52:B52"/>
     <mergeCell ref="A59:B59"/>
     <mergeCell ref="D4:E4"/>

</xml_diff>

<commit_message>
Add projected income section for wife's raise
Co-authored-by: jbox662 <jbox662@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Family_Budget.xlsx
+++ b/Family_Budget.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="97">
   <si>
     <t>MONTHLY BILLS - EDIT HERE</t>
   </si>
@@ -24,7 +24,7 @@
     <t>(Yellow cells are editable - changes update all tabs)</t>
   </si>
   <si>
-    <t>INCOME</t>
+    <t>CURRENT INCOME</t>
   </si>
   <si>
     <t>Source</t>
@@ -39,157 +39,172 @@
     <t>Wife's Income</t>
   </si>
   <si>
+    <t>TOTAL CURRENT INCOME</t>
+  </si>
+  <si>
+    <t>PROJECTED INCOME (After Wife's Raise)</t>
+  </si>
+  <si>
+    <t>Wife's Projected Income</t>
+  </si>
+  <si>
+    <t>TOTAL PROJECTED INCOME</t>
+  </si>
+  <si>
+    <t>PROJECTED INCREASE</t>
+  </si>
+  <si>
+    <t>SETTINGS</t>
+  </si>
+  <si>
+    <t>Bills Account Buffer</t>
+  </si>
+  <si>
+    <t>Monthly Savings Goal</t>
+  </si>
+  <si>
+    <t>VEHICLES</t>
+  </si>
+  <si>
+    <t>Expense</t>
+  </si>
+  <si>
+    <t>Truck Payment</t>
+  </si>
+  <si>
+    <t>Car Payment</t>
+  </si>
+  <si>
+    <t>Boat</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
+    <t>Vehicles Total</t>
+  </si>
+  <si>
+    <t>HOUSING</t>
+  </si>
+  <si>
+    <t>Shelter 1</t>
+  </si>
+  <si>
+    <t>Shelter 2</t>
+  </si>
+  <si>
+    <t>Shelter 3</t>
+  </si>
+  <si>
+    <t>Housing Total</t>
+  </si>
+  <si>
+    <t>UTILITIES</t>
+  </si>
+  <si>
+    <t>Power</t>
+  </si>
+  <si>
+    <t>Internet</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Garbage (Three Rivers)</t>
+  </si>
+  <si>
+    <t>Utilities Total</t>
+  </si>
+  <si>
+    <t>INSURANCE</t>
+  </si>
+  <si>
+    <t>Am Nat</t>
+  </si>
+  <si>
+    <t>Man Life</t>
+  </si>
+  <si>
+    <t>Insurance Total</t>
+  </si>
+  <si>
+    <t>DEBT PAYMENTS</t>
+  </si>
+  <si>
+    <t>IRS</t>
+  </si>
+  <si>
+    <t>Loan (Upstart)</t>
+  </si>
+  <si>
+    <t>Credit Card Consolidation</t>
+  </si>
+  <si>
+    <t>CORS (Wife CC Consolidation)</t>
+  </si>
+  <si>
+    <t>Debt Total</t>
+  </si>
+  <si>
+    <t>OTHER EXPENSES</t>
+  </si>
+  <si>
+    <t>Groceries</t>
+  </si>
+  <si>
+    <t>Shein</t>
+  </si>
+  <si>
+    <t>VB (entry fees)</t>
+  </si>
+  <si>
+    <t>Other Total</t>
+  </si>
+  <si>
+    <t>TOTALS</t>
+  </si>
+  <si>
+    <t>TOTAL ALL EXPENSES</t>
+  </si>
+  <si>
+    <t>CATEGORY SUMMARY</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Vehicles</t>
+  </si>
+  <si>
+    <t>Housing</t>
+  </si>
+  <si>
+    <t>Utilities</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Debt Payments</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>BUDGET OVERVIEW</t>
+  </si>
+  <si>
+    <t>(All values linked to Monthly Bills tab)</t>
+  </si>
+  <si>
     <t>TOTAL INCOME</t>
   </si>
   <si>
-    <t>SETTINGS</t>
-  </si>
-  <si>
-    <t>Bills Account Buffer</t>
-  </si>
-  <si>
-    <t>Monthly Savings Goal</t>
-  </si>
-  <si>
-    <t>VEHICLES</t>
-  </si>
-  <si>
-    <t>Expense</t>
-  </si>
-  <si>
-    <t>Truck Payment</t>
-  </si>
-  <si>
-    <t>Car Payment</t>
-  </si>
-  <si>
-    <t>Boat</t>
-  </si>
-  <si>
-    <t>Fuel</t>
-  </si>
-  <si>
-    <t>Vehicles Total</t>
-  </si>
-  <si>
-    <t>HOUSING</t>
-  </si>
-  <si>
-    <t>Shelter 1</t>
-  </si>
-  <si>
-    <t>Shelter 2</t>
-  </si>
-  <si>
-    <t>Shelter 3</t>
-  </si>
-  <si>
-    <t>Housing Total</t>
-  </si>
-  <si>
-    <t>UTILITIES</t>
-  </si>
-  <si>
-    <t>Power</t>
-  </si>
-  <si>
-    <t>Internet</t>
-  </si>
-  <si>
-    <t>Water</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Garbage (Three Rivers)</t>
-  </si>
-  <si>
-    <t>Utilities Total</t>
-  </si>
-  <si>
-    <t>INSURANCE</t>
-  </si>
-  <si>
-    <t>Am Nat</t>
-  </si>
-  <si>
-    <t>Man Life</t>
-  </si>
-  <si>
-    <t>Insurance Total</t>
-  </si>
-  <si>
-    <t>DEBT PAYMENTS</t>
-  </si>
-  <si>
-    <t>IRS</t>
-  </si>
-  <si>
-    <t>Loan (Upstart)</t>
-  </si>
-  <si>
-    <t>Credit Card Consolidation</t>
-  </si>
-  <si>
-    <t>CORS (Wife CC Consolidation)</t>
-  </si>
-  <si>
-    <t>Debt Total</t>
-  </si>
-  <si>
-    <t>OTHER EXPENSES</t>
-  </si>
-  <si>
-    <t>Groceries</t>
-  </si>
-  <si>
-    <t>Shein</t>
-  </si>
-  <si>
-    <t>VB (entry fees)</t>
-  </si>
-  <si>
-    <t>Other Total</t>
-  </si>
-  <si>
-    <t>TOTALS</t>
-  </si>
-  <si>
-    <t>TOTAL ALL EXPENSES</t>
-  </si>
-  <si>
-    <t>CATEGORY SUMMARY</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Vehicles</t>
-  </si>
-  <si>
-    <t>Housing</t>
-  </si>
-  <si>
-    <t>Utilities</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Debt Payments</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>BUDGET OVERVIEW</t>
-  </si>
-  <si>
-    <t>(All values linked to Monthly Bills tab)</t>
-  </si>
-  <si>
-    <t>ACCOUNT ALLOCATION</t>
+    <t>CURRENT ACCOUNT ALLOCATION</t>
   </si>
   <si>
     <t>Account</t>
@@ -207,7 +222,7 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>MONTHLY SUMMARY</t>
+    <t>CURRENT MONTHLY SUMMARY</t>
   </si>
   <si>
     <t>Total Income</t>
@@ -225,15 +240,33 @@
     <t>Spending Money</t>
   </si>
   <si>
+    <t>PROJECTED INCOME (After Raise)</t>
+  </si>
+  <si>
+    <t>PROJECTED ACCOUNT ALLOCATION</t>
+  </si>
+  <si>
+    <t>PROJECTED MONTHLY SUMMARY</t>
+  </si>
+  <si>
+    <t>Total Projected Income</t>
+  </si>
+  <si>
+    <t>Projected Spending Money</t>
+  </si>
+  <si>
+    <t>EXTRA vs CURRENT</t>
+  </si>
+  <si>
     <t>SPENDING ACCOUNT BUDGET</t>
   </si>
   <si>
+    <t>CURRENT SPENDING BUDGET</t>
+  </si>
+  <si>
     <t>Available for Spending:</t>
   </si>
   <si>
-    <t>(Auto-calculated from Overview)</t>
-  </si>
-  <si>
     <t>Budget</t>
   </si>
   <si>
@@ -267,7 +300,13 @@
     <t>TOTAL BUDGETED</t>
   </si>
   <si>
-    <t>REMAINING UNBUDGETED</t>
+    <t>PROJECTED SPENDING BUDGET</t>
+  </si>
+  <si>
+    <t>Projected Available:</t>
+  </si>
+  <si>
+    <t>EXTRA BUFFER vs CURRENT</t>
   </si>
 </sst>
 </file>
@@ -278,7 +317,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -327,6 +366,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="14"/>
       <color rgb="FF2E7D32"/>
@@ -343,7 +399,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -377,6 +433,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC5E1A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7B68EE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6E6FA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -423,7 +491,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -453,14 +521,31 @@
     <xf numFmtId="164" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -776,7 +861,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>How Your Money Is Split</a:t>
+              <a:t>Current: How Your Money Is Split</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -791,7 +876,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Account Allocation</c:v>
+            <c:v>Current Account Allocation</c:v>
           </c:tx>
           <c:dLbls>
             <c:showCatName val="1"/>
@@ -876,7 +961,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Spending Budget Breakdown</a:t>
+              <a:t>PROJECTED: How Your Money Will Be Split</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -891,7 +976,107 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Spending Budget</c:v>
+            <c:v>Projected Account Allocation</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:showCatName val="1"/>
+            <c:showPercent val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Overview!$D$19:$D$21</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Bills Account</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Savings Account</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Spending Account</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Overview!$E$19:$E$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:style val="10"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Current Spending Breakdown</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Current Spending Budget</c:v>
           </c:tx>
           <c:dLbls>
             <c:showCatName val="1"/>
@@ -955,6 +1140,136 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:style val="10"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>PROJECTED Spending Breakdown</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Projected Spending Budget</c:v>
+          </c:tx>
+          <c:dLbls>
+            <c:showCatName val="1"/>
+            <c:showPercent val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Spending Budget'!$E$7:$E$14</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Dining Out/Entertainment</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Personal (You)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Personal (Wife)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Household Items</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Car Maintenance</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Medical/Health</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Clothing</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Miscellaneous/Buffer</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Spending Budget'!$F$7:$F$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -1061,13 +1376,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>390525</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1087,6 +1402,36 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1094,16 +1439,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>838200</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1117,6 +1462,36 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1410,7 +1785,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -1437,7 +1812,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -1449,7 +1824,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -1463,10 +1838,10 @@
         <v>6000</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="E6" s="8">
-        <f>B20</f>
+        <f>B27</f>
         <v>0</v>
       </c>
     </row>
@@ -1478,10 +1853,10 @@
         <v>4875.5</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E7" s="8">
-        <f>B27</f>
+        <f>B34</f>
         <v>0</v>
       </c>
     </row>
@@ -1494,169 +1869,171 @@
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="E8" s="8">
-        <f>B36</f>
+        <f>B43</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E9" s="8">
-        <f>B42</f>
+        <f>B49</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="3"/>
+      <c r="B10" s="11"/>
       <c r="D10" s="7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E10" s="8">
-        <f>B50</f>
+        <f>B57</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="8">
+        <f>B64</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="13">
+        <f>B6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="6">
-        <v>200</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" s="8">
-        <f>B57</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="5" t="s">
+      <c r="B13" s="13">
+        <v>5875</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="6">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="3" t="s">
+      <c r="B14" s="15">
+        <f>SUM(B12:B13)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="3"/>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="4" t="s">
+      <c r="B15" s="15">
+        <f>B14-B8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="6">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="6">
-        <v>700</v>
-      </c>
+      <c r="B17" s="3"/>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B18" s="6">
-        <v>565</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="6">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="3"/>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="6">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="9" t="s">
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="10">
-        <f>SUM(B16:B19)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" s="3"/>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>4</v>
+      <c r="B23" s="6">
+        <v>900</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B24" s="6">
-        <v>641</v>
+        <v>700</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B25" s="6">
-        <v>362.9</v>
+        <v>565</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B26" s="6">
-        <v>300</v>
+        <v>800</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B27" s="10">
-        <f>SUM(B24:B26)</f>
+        <f>SUM(B23:B26)</f>
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B29" s="3"/>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>4</v>
@@ -1664,221 +2041,269 @@
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B31" s="6">
-        <v>400</v>
+        <v>641</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B32" s="6">
-        <v>85</v>
+        <v>362.9</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" s="6">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B33" s="6">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2">
-      <c r="A34" s="5" t="s">
+      <c r="B34" s="10">
+        <f>SUM(B31:B33)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="6">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2">
-      <c r="A35" s="5" t="s">
+      <c r="B36" s="3"/>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="6">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
-      <c r="A36" s="9" t="s">
+      <c r="B38" s="6">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B36" s="10">
-        <f>SUM(B31:B35)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
-      <c r="A38" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B38" s="3"/>
-    </row>
-    <row r="39" spans="1:2">
-      <c r="A39" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>4</v>
+      <c r="B39" s="6">
+        <v>85</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B40" s="6">
-        <v>104.17</v>
+        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B41" s="6">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B41" s="6">
-        <v>34.3</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2">
-      <c r="A42" s="9" t="s">
+      <c r="B42" s="6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B42" s="10">
-        <f>SUM(B40:B41)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2">
-      <c r="A44" s="3" t="s">
+      <c r="B43" s="10">
+        <f>SUM(B38:B42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B44" s="3"/>
-    </row>
-    <row r="45" spans="1:2">
-      <c r="A45" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3"/>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B46" s="4" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2">
-      <c r="A46" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B46" s="6">
-        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B47" s="6">
-        <v>106.16</v>
+        <v>104.17</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B48" s="6">
+        <v>34.3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B48" s="6">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
-      <c r="A49" s="5" t="s">
+      <c r="B49" s="10">
+        <f>SUM(B47:B48)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B49" s="6">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="A50" s="9" t="s">
+      <c r="B51" s="3"/>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B50" s="10">
-        <f>SUM(B46:B49)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2">
-      <c r="A52" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B52" s="3"/>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>4</v>
+      <c r="B53" s="6">
+        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B54" s="6">
-        <v>600</v>
+        <v>106.16</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B55" s="6">
-        <v>100</v>
+        <v>338</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B56" s="6">
-        <v>240</v>
+        <v>519</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B57" s="10">
-        <f>SUM(B54:B56)</f>
+        <f>SUM(B53:B56)</f>
         <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B59" s="3"/>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B59" s="3"/>
-    </row>
-    <row r="60" spans="1:2">
-      <c r="A60" s="9" t="s">
+      <c r="B61" s="6">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B60" s="10">
-        <f>B20+B27+B36+B42+B50+B57</f>
+      <c r="B62" s="6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B63" s="6">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B64" s="10">
+        <f>SUM(B61:B63)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B66" s="3"/>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B67" s="10">
+        <f>B27+B34+B43+B49+B57+B64</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A21:B21"/>
     <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A51:B51"/>
     <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A66:B66"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1888,7 +2313,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -1900,7 +2325,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1909,7 +2334,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1918,7 +2343,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -1930,7 +2355,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -1945,10 +2370,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="E6" s="8">
-        <f>'Monthly Bills'!B60+'Monthly Bills'!B11</f>
+        <f>'Monthly Bills'!B67+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
     </row>
@@ -1961,23 +2386,23 @@
         <v>0</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="E7" s="8">
-        <f>'Monthly Bills'!B12</f>
+        <f>'Monthly Bills'!B19</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>7</v>
+        <v>61</v>
       </c>
       <c r="B8" s="10">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="E8" s="8">
         <f>'Monthly Bills'!B8-E6-E7</f>
@@ -1986,7 +2411,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="9" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E9" s="10">
         <f>SUM(E6:E8)</f>
@@ -1995,61 +2420,205 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" s="11">
+        <v>69</v>
+      </c>
+      <c r="B11" s="16">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B12" s="12">
-        <f>'Monthly Bills'!B60</f>
+        <v>70</v>
+      </c>
+      <c r="B12" s="17">
+        <f>'Monthly Bills'!B67</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="7" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B13" s="8">
-        <f>'Monthly Bills'!B11</f>
+        <f>'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="7" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B14" s="8">
-        <f>'Monthly Bills'!B12</f>
+        <f>'Monthly Bills'!B19</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B15" s="11">
+        <v>73</v>
+      </c>
+      <c r="B15" s="16">
         <f>E8</f>
         <v>0</v>
       </c>
     </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="11"/>
+      <c r="D17" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" s="11"/>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="13">
+        <f>'Monthly Bills'!B12</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" s="13">
+        <f>'Monthly Bills'!B67+'Monthly Bills'!B18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="13">
+        <f>'Monthly Bills'!B13</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="13">
+        <f>'Monthly Bills'!B19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="15">
+        <f>'Monthly Bills'!B14</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="13">
+        <f>'Monthly Bills'!B14-E19-E20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="D22" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="15">
+        <f>SUM(E19:E21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="11"/>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="13">
+        <f>'Monthly Bills'!B14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" s="13">
+        <f>'Monthly Bills'!B67</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="13">
+        <f>'Monthly Bills'!B18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" s="13">
+        <f>'Monthly Bills'!B19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B28" s="13">
+        <f>E21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" s="15">
+        <f>B28-B15</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="A23:B23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2058,163 +2627,290 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
     <col min="2" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" customWidth="1"/>
+    <col min="6" max="7" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30" customHeight="1">
+    <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3" s="11">
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="E3" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="16">
         <f>Overview!E8</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="E4" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F4" s="13">
+        <f>Overview!E21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <v>84</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="B7" s="6">
         <v>350</v>
       </c>
-      <c r="C7" s="13">
-        <f>IF($B$3&gt;0,B7/$B$3,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="C7" s="18">
+        <f>IF($B$4&gt;0,B7/$B$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="F7" s="13">
+        <f>B7</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="19">
+        <f>IF($F$4&gt;0,F7/$F$4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="5" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="B8" s="6">
         <v>225</v>
       </c>
-      <c r="C8" s="13">
-        <f>IF($B$3&gt;0,B8/$B$3,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="C8" s="18">
+        <f>IF($B$4&gt;0,B8/$B$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" s="13">
+        <f>B8</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="19">
+        <f>IF($F$4&gt;0,F8/$F$4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="B9" s="6">
         <v>225</v>
       </c>
-      <c r="C9" s="13">
-        <f>IF($B$3&gt;0,B9/$B$3,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="C9" s="18">
+        <f>IF($B$4&gt;0,B9/$B$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="F9" s="13">
+        <f>B9</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="19">
+        <f>IF($F$4&gt;0,F9/$F$4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="5" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="B10" s="6">
         <v>175</v>
       </c>
-      <c r="C10" s="13">
-        <f>IF($B$3&gt;0,B10/$B$3,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="C10" s="18">
+        <f>IF($B$4&gt;0,B10/$B$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="F10" s="13">
+        <f>B10</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="19">
+        <f>IF($F$4&gt;0,F10/$F$4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="B11" s="6">
         <v>150</v>
       </c>
-      <c r="C11" s="13">
-        <f>IF($B$3&gt;0,B11/$B$3,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="C11" s="18">
+        <f>IF($B$4&gt;0,B11/$B$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="F11" s="13">
+        <f>B11</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="19">
+        <f>IF($F$4&gt;0,F11/$F$4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="B12" s="6">
         <v>150</v>
       </c>
-      <c r="C12" s="13">
-        <f>IF($B$3&gt;0,B12/$B$3,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="C12" s="18">
+        <f>IF($B$4&gt;0,B12/$B$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F12" s="13">
+        <f>B12</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="19">
+        <f>IF($F$4&gt;0,F12/$F$4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" s="5" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="B13" s="6">
         <v>100</v>
       </c>
-      <c r="C13" s="13">
-        <f>IF($B$3&gt;0,B13/$B$3,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="C13" s="18">
+        <f>IF($B$4&gt;0,B13/$B$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="13">
+        <f>B13</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="19">
+        <f>IF($F$4&gt;0,F13/$F$4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="B14" s="10">
-        <f>$B$3-SUM(B7:B13)</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="14">
-        <f>IF($B$3&gt;0,B14/$B$3,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
+        <f>$B$4-SUM(B7:B13)</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="20">
+        <f>IF($B$4&gt;0,B14/$B$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" s="15">
+        <f>$F$4-SUM(F7:F13)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="21">
+        <f>IF($F$4&gt;0,F14/$F$4,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="B16" s="10">
         <f>SUM(B7:B14)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B17" s="10">
-        <f>$B$3-B16</f>
+      <c r="E16" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="F16" s="15">
+        <f>SUM(F7:F14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="5:6">
+      <c r="E18" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="15">
+        <f>F14-B14</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="E3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Fix: Savings now correctly split between both paychecks (not doubled)
Co-authored-by: jbox662 <jbox662@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Family_Budget.xlsx
+++ b/Family_Budget.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="124">
   <si>
     <t>MONTHLY BILLS - EDIT HERE</t>
   </si>
@@ -205,43 +205,46 @@
     <t>(Shows exactly how much from each paycheck goes to each account)</t>
   </si>
   <si>
-    <t>YOUR PAYCHECKS (15th &amp; Last Day of Month)</t>
+    <t>MONTHLY TARGETS (from Overview)</t>
+  </si>
+  <si>
+    <t>Total Monthly</t>
+  </si>
+  <si>
+    <t>Bills Account</t>
+  </si>
+  <si>
+    <t>Savings Account</t>
+  </si>
+  <si>
+    <t>Spending Account</t>
+  </si>
+  <si>
+    <t>Monthly Target</t>
+  </si>
+  <si>
+    <t>YOUR PAYCHECKS (15th &amp; Last Day of Month) - 2 per month</t>
   </si>
   <si>
     <t>Per Paycheck</t>
   </si>
   <si>
-    <t>Bills Account</t>
-  </si>
-  <si>
-    <t>Savings Account</t>
-  </si>
-  <si>
-    <t>Spending Account</t>
-  </si>
-  <si>
     <t>Your Paycheck Amount</t>
   </si>
   <si>
-    <t>15th Paycheck - Put in:</t>
-  </si>
-  <si>
-    <t>Last Day Paycheck - Put in:</t>
-  </si>
-  <si>
-    <t>YOUR MONTHLY TOTAL</t>
-  </si>
-  <si>
-    <t>WIFE'S PAYCHECKS (Every 2 Weeks - approx 2.17/month)</t>
+    <t>Each Paycheck - Put in:</t>
+  </si>
+  <si>
+    <t>YOUR MONTHLY TOTAL (2 paychecks)</t>
+  </si>
+  <si>
+    <t>WIFE'S PAYCHECKS (Every 2 Weeks) - avg 2.167 per month</t>
   </si>
   <si>
     <t>Wife's Paycheck Amount</t>
   </si>
   <si>
-    <t>Each Paycheck - Put in:</t>
-  </si>
-  <si>
-    <t>WIFE'S MONTHLY TOTAL (avg)</t>
+    <t>WIFE'S MONTHLY TOTAL (avg 2.167 paychecks)</t>
   </si>
   <si>
     <t>COMBINED MONTHLY TOTALS</t>
@@ -253,7 +256,10 @@
     <t>COMBINED MONTHLY</t>
   </si>
   <si>
-    <t>Target from Overview</t>
+    <t>Target (should match)</t>
+  </si>
+  <si>
+    <t>Difference (should be ~$0)</t>
   </si>
   <si>
     <t>QUICK REFERENCE - COPY THIS TO YOUR PHONE!</t>
@@ -2450,7 +2456,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -2472,13 +2478,13 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="4"/>
@@ -2496,320 +2502,366 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="10">
+        <f>'Monthly Bills'!B8</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="10">
+        <f>'Monthly Bills'!B67+'Monthly Bills'!B18</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="10">
+        <f>'Monthly Bills'!B19</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="10">
+        <f>B6-C6-D6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="18">
         <f>'Monthly Bills'!B6/2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="18">
+    <row r="11" spans="1:5">
+      <c r="A11" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="18">
+        <f>B10</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="18">
+        <f>ROUND(('Monthly Bills'!B6/'Monthly Bills'!B8)*$C$6/2,2)</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="18">
+        <f>ROUND(('Monthly Bills'!B6/'Monthly Bills'!B8)*$D$6/2,2)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="18">
+        <f>B11-C11-D11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" s="20">
+        <f>B11*2</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="20">
+        <f>C11*2</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="20">
+        <f>D11*2</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="20">
+        <f>E11*2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="18">
+        <f>'Monthly Bills'!B7/2.167</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="18">
+        <f>B16</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="18">
+        <f>ROUND(('Monthly Bills'!B7/'Monthly Bills'!B8)*$C$6/2.167,2)</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="18">
+        <f>ROUND(('Monthly Bills'!B7/'Monthly Bills'!B8)*$D$6/2.167,2)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="18">
+        <f>B17-C17-D17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="20">
+        <f>B17*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="20">
+        <f>C17*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="20">
+        <f>D17*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="20">
+        <f>E17*2.167</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="10">
+        <f>B12+B18</f>
+        <v>0</v>
+      </c>
+      <c r="C22" s="10">
+        <f>C12+C18</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="10">
+        <f>D12+D18</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="10">
+        <f>E12+E18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="8">
         <f>B6</f>
         <v>0</v>
       </c>
-      <c r="C7" s="18">
-        <f>ROUND(('Monthly Bills'!B67+'Monthly Bills'!B18)*(B6/'Monthly Bills'!B8),2)</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="18">
-        <f>ROUND('Monthly Bills'!B19/2,2)</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="18">
-        <f>B7-C7-D7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="18">
-        <f>B6</f>
-        <v>0</v>
-      </c>
-      <c r="C8" s="18">
-        <f>C7</f>
-        <v>0</v>
-      </c>
-      <c r="D8" s="18">
-        <f>D7</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="18">
-        <f>B8-C8-D8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="B9" s="20">
-        <f>B7+B8</f>
-        <v>0</v>
-      </c>
-      <c r="C9" s="20">
-        <f>C7+C8</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="20">
-        <f>D7+D8</f>
-        <v>0</v>
-      </c>
-      <c r="E9" s="20">
-        <f>E7+E8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B13" s="18">
-        <f>'Monthly Bills'!B7/2.167</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="18">
-        <f>B13</f>
-        <v>0</v>
-      </c>
-      <c r="C14" s="18">
-        <f>ROUND(('Monthly Bills'!B67+'Monthly Bills'!B18)*(B13*2.167/'Monthly Bills'!B8)/2.167,2)</f>
-        <v>0</v>
-      </c>
-      <c r="D14" s="18">
-        <f>ROUND('Monthly Bills'!B19/2.167,2)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="18">
-        <f>B14-C14-D14</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="20">
-        <f>B14*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="20">
-        <f>C14*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="20">
-        <f>D14*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="20">
-        <f>E14*2.167</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B19" s="10">
-        <f>B9+B15</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="10">
-        <f>C9+C15</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="10">
-        <f>D9+D15</f>
-        <v>0</v>
-      </c>
-      <c r="E19" s="10">
-        <f>E9+E15</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="B20" s="8">
-        <f>'Monthly Bills'!B8</f>
-        <v>0</v>
-      </c>
-      <c r="C20" s="8">
-        <f>'Monthly Bills'!B67+'Monthly Bills'!B18</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="8">
-        <f>'Monthly Bills'!B19</f>
-        <v>0</v>
-      </c>
-      <c r="E20" s="8">
-        <f>B20-C20-D20</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
+      <c r="C23" s="8">
+        <f>C6</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="8">
+        <f>D6</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="8">
+        <f>E6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B24" s="16"/>
-      <c r="D24" s="16" t="s">
+      <c r="B24" s="8">
+        <f>B22-B23</f>
+        <v>0</v>
+      </c>
+      <c r="C24" s="8">
+        <f>C22-C23</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="8">
+        <f>D22-D23</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="8">
+        <f>E22-E23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" s="16"/>
+      <c r="D28" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="E28" s="16"/>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B29" s="20">
+        <f>C11</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="E29" s="20">
+        <f>C17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B30" s="20">
+        <f>D11</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="20">
+        <f>D17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="E24" s="16"/>
-    </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="B25" s="20">
-        <f>C7</f>
-        <v>0</v>
-      </c>
-      <c r="D25" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="E25" s="20">
-        <f>C14</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="B26" s="20">
-        <f>D7</f>
-        <v>0</v>
-      </c>
-      <c r="D26" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="E26" s="20">
-        <f>D14</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="B27" s="20">
-        <f>E7</f>
-        <v>0</v>
-      </c>
-      <c r="D27" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="E27" s="20">
-        <f>E14</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="B28" s="20">
-        <f>B6</f>
-        <v>0</v>
-      </c>
-      <c r="D28" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="E28" s="20">
-        <f>B13</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="22" t="s">
+      <c r="B31" s="20">
+        <f>E11</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E31" s="20">
+        <f>E17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
+      <c r="B32" s="20">
+        <f>B10</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="E32" s="20">
+        <f>B16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="22"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="A34:E34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2829,7 +2881,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2838,7 +2890,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2847,7 +2899,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -2859,7 +2911,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -2883,7 +2935,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B7" s="8">
         <f>'Monthly Bills'!B7</f>
@@ -2899,7 +2951,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B8" s="10">
         <f>'Monthly Bills'!B8</f>
@@ -2915,7 +2967,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E9" s="10">
         <f>SUM(E6:E8)</f>
@@ -2924,13 +2976,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B11" s="23">
         <f>'Monthly Bills'!B8</f>
@@ -2939,7 +2991,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B12" s="24">
         <f>'Monthly Bills'!B67</f>
@@ -2948,7 +3000,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B13" s="8">
         <f>'Monthly Bills'!B18</f>
@@ -2957,7 +3009,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B14" s="8">
         <f>'Monthly Bills'!B19</f>
@@ -2966,7 +3018,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B15" s="23">
         <f>E8</f>
@@ -2975,11 +3027,11 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B17" s="11"/>
       <c r="D17" s="11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E17" s="11"/>
     </row>
@@ -2991,7 +3043,7 @@
         <v>4</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>4</v>
@@ -3047,7 +3099,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="D22" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E22" s="15">
         <f>SUM(E19:E21)</f>
@@ -3056,13 +3108,13 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B23" s="11"/>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B24" s="13">
         <f>'Monthly Bills'!B14</f>
@@ -3071,7 +3123,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B25" s="13">
         <f>'Monthly Bills'!B67</f>
@@ -3080,7 +3132,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="12" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B26" s="13">
         <f>'Monthly Bills'!B18</f>
@@ -3089,7 +3141,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B27" s="13">
         <f>'Monthly Bills'!B19</f>
@@ -3098,7 +3150,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B28" s="13">
         <f>E21</f>
@@ -3107,7 +3159,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="14" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B29" s="15">
         <f>B28-B15</f>
@@ -3143,7 +3195,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3154,26 +3206,26 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" s="11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B4" s="23">
         <f>Overview!E8</f>
         <v>0</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F4" s="13">
         <f>Overview!E21</f>
@@ -3185,24 +3237,24 @@
         <v>53</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>53</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B7" s="6">
         <v>350</v>
@@ -3212,7 +3264,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F7" s="13">
         <f>B7</f>
@@ -3225,7 +3277,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B8" s="6">
         <v>225</v>
@@ -3235,7 +3287,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F8" s="13">
         <f>B8</f>
@@ -3248,7 +3300,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B9" s="6">
         <v>225</v>
@@ -3258,7 +3310,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F9" s="13">
         <f>B9</f>
@@ -3271,7 +3323,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B10" s="6">
         <v>175</v>
@@ -3281,7 +3333,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F10" s="13">
         <f>B10</f>
@@ -3294,7 +3346,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B11" s="6">
         <v>150</v>
@@ -3304,7 +3356,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F11" s="13">
         <f>B11</f>
@@ -3317,7 +3369,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B12" s="6">
         <v>150</v>
@@ -3327,7 +3379,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F12" s="13">
         <f>B12</f>
@@ -3340,7 +3392,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B13" s="6">
         <v>100</v>
@@ -3350,7 +3402,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F13" s="13">
         <f>B13</f>
@@ -3363,7 +3415,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B14" s="10">
         <f>$B$4-SUM(B7:B13)</f>
@@ -3374,7 +3426,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F14" s="15">
         <f>$F$4-SUM(F7:F13)</f>
@@ -3387,14 +3439,14 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B16" s="10">
         <f>SUM(B7:B14)</f>
         <v>0</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F16" s="15">
         <f>SUM(F7:F14)</f>
@@ -3403,7 +3455,7 @@
     </row>
     <row r="18" spans="5:6">
       <c r="E18" s="14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F18" s="15">
         <f>F14-B14</f>

</xml_diff>

<commit_message>
Fix: Savings correctly split - Your share ~96/mo, Wife share ~03/mo = 00 total
Co-authored-by: jbox662 <jbox662@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Family_Budget.xlsx
+++ b/Family_Budget.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="126">
   <si>
     <t>MONTHLY BILLS - EDIT HERE</t>
   </si>
@@ -205,7 +205,7 @@
     <t>(Shows exactly how much from each paycheck goes to each account)</t>
   </si>
   <si>
-    <t>MONTHLY TARGETS (from Overview)</t>
+    <t>MONTHLY TARGETS (what we need total each month)</t>
   </si>
   <si>
     <t>Total Monthly</t>
@@ -232,22 +232,28 @@
     <t>Your Paycheck Amount</t>
   </si>
   <si>
+    <t>15th Paycheck - Put in:</t>
+  </si>
+  <si>
+    <t>Last Day Paycheck - Put in:</t>
+  </si>
+  <si>
+    <t>YOUR MONTHLY TOTAL</t>
+  </si>
+  <si>
+    <t>WIFE'S PAYCHECKS (Every 2 Weeks) - avg 2.167 per month</t>
+  </si>
+  <si>
+    <t>Wife's Paycheck Amount</t>
+  </si>
+  <si>
     <t>Each Paycheck - Put in:</t>
   </si>
   <si>
-    <t>YOUR MONTHLY TOTAL (2 paychecks)</t>
-  </si>
-  <si>
-    <t>WIFE'S PAYCHECKS (Every 2 Weeks) - avg 2.167 per month</t>
-  </si>
-  <si>
-    <t>Wife's Paycheck Amount</t>
-  </si>
-  <si>
-    <t>WIFE'S MONTHLY TOTAL (avg 2.167 paychecks)</t>
-  </si>
-  <si>
-    <t>COMBINED MONTHLY TOTALS</t>
+    <t>WIFE'S MONTHLY TOTAL (avg)</t>
+  </si>
+  <si>
+    <t>COMBINED MONTHLY TOTALS (You + Wife)</t>
   </si>
   <si>
     <t>Total Income</t>
@@ -2456,7 +2462,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -2577,291 +2583,312 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="20">
-        <f>B11*2</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="20">
-        <f>C11*2</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="20">
-        <f>D11*2</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="20">
-        <f>E11*2</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="16" t="s">
+      <c r="B12" s="18">
+        <f>B10</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="18">
+        <f>C11</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="18">
+        <f>D11</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="18">
+        <f>E11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
+      <c r="B13" s="20">
+        <f>B11+B12</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="20">
+        <f>C11+C12</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="20">
+        <f>D11+D12</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="20">
+        <f>E11+E12</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>66</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="B16" s="18">
-        <f>'Monthly Bills'!B7/2.167</f>
-        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B17" s="18">
-        <f>B16</f>
-        <v>0</v>
-      </c>
-      <c r="C17" s="18">
+        <f>'Monthly Bills'!B7/2.167</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="18">
+        <f>B17</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="18">
         <f>ROUND(('Monthly Bills'!B7/'Monthly Bills'!B8)*$C$6/2.167,2)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="18">
+      <c r="D18" s="18">
         <f>ROUND(('Monthly Bills'!B7/'Monthly Bills'!B8)*$D$6/2.167,2)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="18">
-        <f>B17-C17-D17</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="20">
-        <f>B17*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="C18" s="20">
-        <f>C17*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="20">
-        <f>D17*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="20">
-        <f>E17*2.167</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
+      <c r="E18" s="18">
+        <f>B18-C18-D18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="20">
+        <f>B18*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="20">
+        <f>C18*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="20">
+        <f>D18*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="20">
+        <f>E18*2.167</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="A21" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D22" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" s="10">
-        <f>B12+B18</f>
-        <v>0</v>
-      </c>
-      <c r="C22" s="10">
-        <f>C12+C18</f>
-        <v>0</v>
-      </c>
-      <c r="D22" s="10">
-        <f>D12+D18</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="10">
-        <f>E12+E18</f>
-        <v>0</v>
-      </c>
-    </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="B23" s="8">
-        <f>B6</f>
-        <v>0</v>
-      </c>
-      <c r="C23" s="8">
-        <f>C6</f>
-        <v>0</v>
-      </c>
-      <c r="D23" s="8">
-        <f>D6</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="8">
-        <f>E6</f>
+      <c r="A23" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" s="10">
+        <f>B13+B19</f>
+        <v>0</v>
+      </c>
+      <c r="C23" s="10">
+        <f>C13+C19</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="10">
+        <f>D13+D19</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="10">
+        <f>E13+E19</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B24" s="8">
-        <f>B22-B23</f>
+        <f>B6</f>
         <v>0</v>
       </c>
       <c r="C24" s="8">
-        <f>C22-C23</f>
+        <f>C6</f>
         <v>0</v>
       </c>
       <c r="D24" s="8">
-        <f>D22-D23</f>
+        <f>D6</f>
         <v>0</v>
       </c>
       <c r="E24" s="8">
-        <f>E22-E23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
-      <c r="A26" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="B26" s="21"/>
-      <c r="C26" s="21"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-    </row>
-    <row r="28" spans="1:5">
-      <c r="A28" s="16" t="s">
+        <f>E6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B28" s="16"/>
-      <c r="D28" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="E28" s="16"/>
+      <c r="B25" s="8">
+        <f>B23-B24</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="8">
+        <f>C23-C24</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="8">
+        <f>D23-D24</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="8">
+        <f>E23-E24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="B29" s="20">
-        <f>C11</f>
-        <v>0</v>
-      </c>
-      <c r="D29" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="E29" s="20">
-        <f>C17</f>
-        <v>0</v>
-      </c>
+      <c r="A29" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" s="16"/>
+      <c r="D29" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="E29" s="16"/>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B30" s="20">
-        <f>D11</f>
+        <f>C11</f>
         <v>0</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E30" s="20">
-        <f>D17</f>
+        <f>C18</f>
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B31" s="20">
+        <f>D11</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="E31" s="20">
+        <f>D18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="20">
         <f>E11</f>
         <v>0</v>
       </c>
-      <c r="D31" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="E31" s="20">
-        <f>E17</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="B32" s="20">
+      <c r="D32" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E32" s="20">
+        <f>E18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B33" s="20">
         <f>B10</f>
         <v>0</v>
       </c>
-      <c r="D32" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="E32" s="20">
-        <f>B16</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="22" t="s">
+      <c r="D33" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="B34" s="22"/>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
+      <c r="E33" s="20">
+        <f>B17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="22"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A35:E35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2881,7 +2908,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2890,7 +2917,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2899,7 +2926,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -2911,7 +2938,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -2935,7 +2962,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B7" s="8">
         <f>'Monthly Bills'!B7</f>
@@ -2951,7 +2978,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B8" s="10">
         <f>'Monthly Bills'!B8</f>
@@ -2967,7 +2994,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E9" s="10">
         <f>SUM(E6:E8)</f>
@@ -2976,13 +3003,13 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B10" s="3"/>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B11" s="23">
         <f>'Monthly Bills'!B8</f>
@@ -2991,7 +3018,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B12" s="24">
         <f>'Monthly Bills'!B67</f>
@@ -3000,7 +3027,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B13" s="8">
         <f>'Monthly Bills'!B18</f>
@@ -3009,7 +3036,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B14" s="8">
         <f>'Monthly Bills'!B19</f>
@@ -3018,7 +3045,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B15" s="23">
         <f>E8</f>
@@ -3027,11 +3054,11 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B17" s="11"/>
       <c r="D17" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E17" s="11"/>
     </row>
@@ -3043,7 +3070,7 @@
         <v>4</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>4</v>
@@ -3099,7 +3126,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="D22" s="14" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E22" s="15">
         <f>SUM(E19:E21)</f>
@@ -3108,13 +3135,13 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B23" s="11"/>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B24" s="13">
         <f>'Monthly Bills'!B14</f>
@@ -3123,7 +3150,7 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B25" s="13">
         <f>'Monthly Bills'!B67</f>
@@ -3132,7 +3159,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B26" s="13">
         <f>'Monthly Bills'!B18</f>
@@ -3141,7 +3168,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B27" s="13">
         <f>'Monthly Bills'!B19</f>
@@ -3150,7 +3177,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B28" s="13">
         <f>E21</f>
@@ -3159,7 +3186,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="14" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B29" s="15">
         <f>B28-B15</f>
@@ -3195,7 +3222,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3206,26 +3233,26 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" s="11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B4" s="23">
         <f>Overview!E8</f>
         <v>0</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F4" s="13">
         <f>Overview!E21</f>
@@ -3237,24 +3264,24 @@
         <v>53</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>53</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B7" s="6">
         <v>350</v>
@@ -3264,7 +3291,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F7" s="13">
         <f>B7</f>
@@ -3277,7 +3304,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B8" s="6">
         <v>225</v>
@@ -3287,7 +3314,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F8" s="13">
         <f>B8</f>
@@ -3300,7 +3327,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B9" s="6">
         <v>225</v>
@@ -3310,7 +3337,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F9" s="13">
         <f>B9</f>
@@ -3323,7 +3350,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B10" s="6">
         <v>175</v>
@@ -3333,7 +3360,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F10" s="13">
         <f>B10</f>
@@ -3346,7 +3373,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B11" s="6">
         <v>150</v>
@@ -3356,7 +3383,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F11" s="13">
         <f>B11</f>
@@ -3369,7 +3396,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B12" s="6">
         <v>150</v>
@@ -3379,7 +3406,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F12" s="13">
         <f>B12</f>
@@ -3392,7 +3419,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B13" s="6">
         <v>100</v>
@@ -3402,7 +3429,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F13" s="13">
         <f>B13</f>
@@ -3415,7 +3442,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B14" s="10">
         <f>$B$4-SUM(B7:B13)</f>
@@ -3426,7 +3453,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F14" s="15">
         <f>$F$4-SUM(F7:F13)</f>
@@ -3439,14 +3466,14 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B16" s="10">
         <f>SUM(B7:B14)</f>
         <v>0</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F16" s="15">
         <f>SUM(F7:F14)</f>
@@ -3455,7 +3482,7 @@
     </row>
     <row r="18" spans="5:6">
       <c r="E18" s="14" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F18" s="15">
         <f>F14-B14</f>

</xml_diff>

<commit_message>
Add direct deposit section - 50/check for boat & loan auto-deducted
Co-authored-by: jbox662 <jbox662@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Family_Budget.xlsx
+++ b/Family_Budget.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="143">
   <si>
     <t>MONTHLY BILLS - EDIT HERE</t>
   </si>
@@ -67,6 +67,27 @@
     <t>Monthly Savings Goal</t>
   </si>
   <si>
+    <t>DIRECT DEPOSIT (Auto-deducted from paycheck)</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Per Paycheck</t>
+  </si>
+  <si>
+    <t>Your DD (Boat &amp; Small Loan)</t>
+  </si>
+  <si>
+    <t>Wife's DD (if any)</t>
+  </si>
+  <si>
+    <t>Your Monthly DD Total</t>
+  </si>
+  <si>
+    <t>Wife's Monthly DD Total</t>
+  </si>
+  <si>
     <t>VEHICLES</t>
   </si>
   <si>
@@ -79,7 +100,7 @@
     <t>Car Payment</t>
   </si>
   <si>
-    <t>Boat</t>
+    <t>Boat (via Direct Deposit)</t>
   </si>
   <si>
     <t>Fuel</t>
@@ -175,6 +196,12 @@
     <t>TOTAL ALL EXPENSES</t>
   </si>
   <si>
+    <t>Paid via Direct Deposit</t>
+  </si>
+  <si>
+    <t>Remaining to pay from accounts</t>
+  </si>
+  <si>
     <t>CATEGORY SUMMARY</t>
   </si>
   <si>
@@ -226,28 +253,34 @@
     <t>YOUR PAYCHECKS (15th &amp; Last Day of Month) - 2 per month</t>
   </si>
   <si>
-    <t>Per Paycheck</t>
-  </si>
-  <si>
-    <t>Your Paycheck Amount</t>
-  </si>
-  <si>
-    <t>15th Paycheck - Put in:</t>
-  </si>
-  <si>
-    <t>Last Day Paycheck - Put in:</t>
+    <t>Your Gross Paycheck</t>
+  </si>
+  <si>
+    <t>MINUS: Direct Deposit (Boat &amp; Loan)</t>
+  </si>
+  <si>
+    <t>Your Take-Home to Split</t>
+  </si>
+  <si>
+    <t>Each Paycheck - Put in:</t>
   </si>
   <si>
     <t>YOUR MONTHLY TOTAL</t>
   </si>
   <si>
+    <t>(Plus Direct Deposit pays bills)</t>
+  </si>
+  <si>
     <t>WIFE'S PAYCHECKS (Every 2 Weeks) - avg 2.167 per month</t>
   </si>
   <si>
-    <t>Wife's Paycheck Amount</t>
-  </si>
-  <si>
-    <t>Each Paycheck - Put in:</t>
+    <t>Wife's Gross Paycheck</t>
+  </si>
+  <si>
+    <t>MINUS: Direct Deposit (if any)</t>
+  </si>
+  <si>
+    <t>Wife's Take-Home to Split</t>
   </si>
   <si>
     <t>WIFE'S MONTHLY TOTAL (avg)</t>
@@ -259,37 +292,52 @@
     <t>Total Income</t>
   </si>
   <si>
-    <t>COMBINED MONTHLY</t>
+    <t>From Paychecks to Accounts</t>
+  </si>
+  <si>
+    <t>Direct Deposits (pay bills directly)</t>
+  </si>
+  <si>
+    <t>(pays bills)</t>
+  </si>
+  <si>
+    <t>GRAND TOTAL</t>
   </si>
   <si>
     <t>Target (should match)</t>
   </si>
   <si>
-    <t>Difference (should be ~$0)</t>
-  </si>
-  <si>
     <t>QUICK REFERENCE - COPY THIS TO YOUR PHONE!</t>
   </si>
   <si>
     <t>YOUR PAYCHECKS (15th &amp; Last Day)</t>
   </si>
   <si>
-    <t>Bills Account:</t>
-  </si>
-  <si>
-    <t>Savings Account:</t>
-  </si>
-  <si>
-    <t>Spending Account:</t>
-  </si>
-  <si>
-    <t>TOTAL:</t>
+    <t>Gross Paycheck:</t>
+  </si>
+  <si>
+    <t>Direct Deposit (auto):</t>
+  </si>
+  <si>
+    <t>Take-Home to Split:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  → Bills Account:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  → Savings Account:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  → Spending Account:</t>
   </si>
   <si>
     <t>WIFE'S PAYCHECKS (Every 2 Weeks)</t>
   </si>
   <si>
-    <t>NOTE: Wife gets 3 paychecks some months (2 extra/year). Use those for extra savings or debt payoff!</t>
+    <t>NOTE: Your $450 direct deposit automatically pays Boat &amp; Small Loan - already accounted for in bills!</t>
+  </si>
+  <si>
+    <t>Wife gets 3 paychecks some months (2 extra/year). Use those for extra savings or debt payoff!</t>
   </si>
   <si>
     <t>BUDGET OVERVIEW</t>
@@ -308,6 +356,9 @@
   </si>
   <si>
     <t>Account</t>
+  </si>
+  <si>
+    <t>Direct Deposits (auto)</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -405,7 +456,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -479,6 +530,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFDC143C"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF666666"/>
@@ -503,7 +563,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -554,6 +614,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFDC143C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF20B2AA"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -561,6 +627,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE0FFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE4E1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -619,7 +691,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -667,28 +739,40 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1033,9 +1117,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Overview!$D$6:$D$8</c:f>
+              <c:f>Overview!$D$6:$D$9</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>Bills Account</c:v>
                 </c:pt>
@@ -1044,16 +1128,19 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Spending Account</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Direct Deposits (auto)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Overview!$E$6:$E$8</c:f>
+              <c:f>Overview!$E$6:$E$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1061,6 +1148,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1133,9 +1223,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Overview!$D$19:$D$21</c:f>
+              <c:f>Overview!$D$19:$D$22</c:f>
               <c:strCache>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>Bills Account</c:v>
                 </c:pt>
@@ -1144,16 +1234,19 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Spending Account</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Direct Deposits (auto)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Overview!$E$19:$E$21</c:f>
+              <c:f>Overview!$E$19:$E$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1161,6 +1254,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1525,13 +1621,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>390525</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>38</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1555,13 +1651,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>390525</xdr:colOff>
-      <xdr:row>53</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1934,7 +2030,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -1961,7 +2057,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -1973,7 +2069,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -1987,10 +2083,10 @@
         <v>6000</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="E6" s="8">
-        <f>B27</f>
+        <f>B34</f>
         <v>0</v>
       </c>
     </row>
@@ -2002,10 +2098,10 @@
         <v>4875.5</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="E7" s="8">
-        <f>B34</f>
+        <f>B41</f>
         <v>0</v>
       </c>
     </row>
@@ -2018,19 +2114,19 @@
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E8" s="8">
-        <f>B43</f>
+        <f>B50</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="7" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="E9" s="8">
-        <f>B49</f>
+        <f>B56</f>
         <v>0</v>
       </c>
     </row>
@@ -2040,10 +2136,10 @@
       </c>
       <c r="B10" s="11"/>
       <c r="D10" s="7" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E10" s="8">
-        <f>B57</f>
+        <f>B64</f>
         <v>0</v>
       </c>
     </row>
@@ -2055,10 +2151,10 @@
         <v>4</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E11" s="8">
-        <f>B64</f>
+        <f>B71</f>
         <v>0</v>
       </c>
     </row>
@@ -2120,116 +2216,117 @@
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="3"/>
+      <c r="B21" s="16"/>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="6">
-        <v>900</v>
+        <v>450</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B24" s="6">
-        <v>700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" s="6">
-        <v>565</v>
+      <c r="A25" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="10">
+        <f>B23*2</f>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B26" s="6">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
-      <c r="A27" s="9" t="s">
+      <c r="A26" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B27" s="10">
-        <f>SUM(B23:B26)</f>
-        <v>0</v>
-      </c>
+      <c r="B26" s="10">
+        <f>B24*2.167</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="3"/>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" s="3"/>
+      <c r="A29" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>4</v>
+      <c r="A30" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="6">
+        <v>900</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B31" s="6">
-        <v>641</v>
+        <v>700</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B32" s="6">
-        <v>362.9</v>
+        <v>565</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B33" s="6">
-        <v>300</v>
+        <v>800</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B34" s="10">
-        <f>SUM(B31:B33)</f>
+        <f>SUM(B30:B33)</f>
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B36" s="3"/>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>4</v>
@@ -2237,222 +2334,288 @@
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B38" s="6">
-        <v>400</v>
+        <v>641</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B39" s="6">
-        <v>85</v>
+        <v>362.9</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B40" s="6">
-        <v>120</v>
+        <v>300</v>
       </c>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B41" s="6">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2">
-      <c r="A42" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B42" s="6">
-        <v>14</v>
+      <c r="A41" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B41" s="10">
+        <f>SUM(B38:B40)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B43" s="10">
-        <f>SUM(B38:B42)</f>
-        <v>0</v>
+      <c r="A43" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B43" s="3"/>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B45" s="3"/>
+      <c r="A45" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B45" s="6">
+        <v>400</v>
+      </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>4</v>
+      <c r="A46" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B46" s="6">
+        <v>85</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B47" s="6">
-        <v>104.17</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B48" s="6">
-        <v>34.3</v>
+        <v>550</v>
       </c>
     </row>
     <row r="49" spans="1:2">
-      <c r="A49" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B49" s="10">
-        <f>SUM(B47:B48)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2">
-      <c r="A51" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B51" s="3"/>
+      <c r="A49" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" s="6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B50" s="10">
+        <f>SUM(B45:B49)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="52" spans="1:2">
-      <c r="A52" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B52" s="4" t="s">
+      <c r="A52" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B52" s="3"/>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B53" s="4" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B53" s="6">
-        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B54" s="6">
-        <v>106.16</v>
+        <v>104.17</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B55" s="6">
-        <v>338</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="56" spans="1:2">
-      <c r="A56" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B56" s="6">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2">
-      <c r="A57" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B57" s="10">
-        <f>SUM(B53:B56)</f>
-        <v>0</v>
-      </c>
+      <c r="A56" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B56" s="10">
+        <f>SUM(B54:B55)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B58" s="3"/>
     </row>
     <row r="59" spans="1:2">
-      <c r="A59" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B59" s="3"/>
+      <c r="A59" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="60" spans="1:2">
-      <c r="A60" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>4</v>
+      <c r="A60" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B60" s="6">
+        <v>105</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B61" s="6">
-        <v>600</v>
+        <v>106.16</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B62" s="6">
-        <v>100</v>
+        <v>338</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B63" s="6">
-        <v>240</v>
+        <v>519</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B64" s="10">
-        <f>SUM(B61:B63)</f>
+        <f>SUM(B60:B63)</f>
         <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B66" s="3"/>
     </row>
     <row r="67" spans="1:2">
-      <c r="A67" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B67" s="10">
-        <f>B27+B34+B43+B49+B57+B64</f>
+      <c r="A67" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B68" s="6">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B69" s="6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B70" s="6">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B71" s="10">
+        <f>SUM(B68:B70)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B73" s="3"/>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B74" s="10">
+        <f>B34+B41+B50+B56+B64+B71</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B75" s="8">
+        <f>B25+B26</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B76" s="10">
+        <f>B74-B75</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A58:B58"/>
     <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A73:B73"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2462,16 +2625,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="1" max="1" width="40.7109375" customWidth="1"/>
     <col min="2" max="5" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2480,12 +2643,12 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -2495,28 +2658,28 @@
     <row r="5" spans="1:5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="B6" s="10">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
       <c r="C6" s="10">
-        <f>'Monthly Bills'!B67+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B76+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
       <c r="D6" s="10">
@@ -2524,371 +2687,458 @@
         <v>0</v>
       </c>
       <c r="E6" s="10">
-        <f>B6-C6-D6</f>
+        <f>B6-C6-D6-'Monthly Bills'!B25-'Monthly Bills'!B26</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
+      <c r="A8" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="4"/>
       <c r="B9" s="4" t="s">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="B10" s="18">
+      <c r="A10" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="19">
         <f>'Monthly Bills'!B6/2</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="B11" s="18">
-        <f>B10</f>
-        <v>0</v>
-      </c>
-      <c r="C11" s="18">
+      <c r="A11" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="21">
+        <f>-'Monthly Bills'!B23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="23">
+        <f>B10+B11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="19">
+        <f>B12</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="19">
         <f>ROUND(('Monthly Bills'!B6/'Monthly Bills'!B8)*$C$6/2,2)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D13" s="19">
         <f>ROUND(('Monthly Bills'!B6/'Monthly Bills'!B8)*$D$6/2,2)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="18">
-        <f>B11-C11-D11</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="18">
-        <f>B10</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="18">
-        <f>C11</f>
-        <v>0</v>
-      </c>
-      <c r="D12" s="18">
-        <f>D11</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="18">
-        <f>E11</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="B13" s="20">
-        <f>B11+B12</f>
-        <v>0</v>
-      </c>
-      <c r="C13" s="20">
-        <f>C11+C12</f>
-        <v>0</v>
-      </c>
-      <c r="D13" s="20">
-        <f>D11+D12</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="20">
-        <f>E11+E12</f>
+      <c r="E13" s="19">
+        <f>B13-C13-D13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="23">
+        <f>B13*2</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="23">
+        <f>C13*2</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="23">
+        <f>D13*2</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="23">
+        <f>E13*2</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>66</v>
+      <c r="A15" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="21">
+        <f>'Monthly Bills'!B25</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B17" s="18">
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="19">
         <f>'Monthly Bills'!B7/2.167</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="18">
-        <f>B17</f>
-        <v>0</v>
-      </c>
-      <c r="C18" s="18">
+    <row r="20" spans="1:5">
+      <c r="A20" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" s="21">
+        <f>-'Monthly Bills'!B24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="23">
+        <f>B19+B20</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="19">
+        <f>B21</f>
+        <v>0</v>
+      </c>
+      <c r="C22" s="19">
         <f>ROUND(('Monthly Bills'!B7/'Monthly Bills'!B8)*$C$6/2.167,2)</f>
         <v>0</v>
       </c>
-      <c r="D18" s="18">
+      <c r="D22" s="19">
         <f>ROUND(('Monthly Bills'!B7/'Monthly Bills'!B8)*$D$6/2.167,2)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="18">
-        <f>B18-C18-D18</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
-      <c r="A19" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="B19" s="20">
-        <f>B18*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="C19" s="20">
-        <f>C18*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="20">
-        <f>D18*2.167</f>
-        <v>0</v>
-      </c>
-      <c r="E19" s="20">
-        <f>E18*2.167</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
-      <c r="A21" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>66</v>
+      <c r="E22" s="19">
+        <f>B22-C22-D22</f>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" s="10">
-        <f>B13+B19</f>
-        <v>0</v>
-      </c>
-      <c r="C23" s="10">
-        <f>C13+C19</f>
-        <v>0</v>
-      </c>
-      <c r="D23" s="10">
-        <f>D13+D19</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="10">
-        <f>E13+E19</f>
+      <c r="A23" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="23">
+        <f>B22*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="C23" s="23">
+        <f>C22*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="23">
+        <f>D22*2.167</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="23">
+        <f>E22*2.167</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="B24" s="8">
+      <c r="A24" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B24" s="21">
+        <f>'Monthly Bills'!B26</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" s="10">
+        <f>B14+B23</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="10">
+        <f>C14+C23</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="10">
+        <f>D14+D23</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="10">
+        <f>E14+E23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="B29" s="21">
+        <f>B15+B24</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="23">
+        <f>B28+B29</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="23">
+        <f>C28</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="23">
+        <f>D28</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="23">
+        <f>E28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B31" s="8">
         <f>B6</f>
         <v>0</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C31" s="8">
         <f>C6</f>
         <v>0</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D31" s="8">
         <f>D6</f>
         <v>0</v>
       </c>
-      <c r="E24" s="8">
+      <c r="E31" s="8">
         <f>E6</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
-      <c r="A25" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="B25" s="8">
-        <f>B23-B24</f>
-        <v>0</v>
-      </c>
-      <c r="C25" s="8">
-        <f>C23-C24</f>
-        <v>0</v>
-      </c>
-      <c r="D25" s="8">
-        <f>D23-D24</f>
-        <v>0</v>
-      </c>
-      <c r="E25" s="8">
-        <f>E23-E24</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
-      <c r="A27" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B29" s="16"/>
-      <c r="D29" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="E29" s="16"/>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="B30" s="20">
-        <f>C11</f>
-        <v>0</v>
-      </c>
-      <c r="D30" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="E30" s="20">
-        <f>C18</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5">
-      <c r="A31" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="B31" s="20">
-        <f>D11</f>
-        <v>0</v>
-      </c>
-      <c r="D31" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="E31" s="20">
-        <f>D18</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
-      <c r="A32" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="B32" s="20">
-        <f>E11</f>
-        <v>0</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E32" s="20">
-        <f>E18</f>
-        <v>0</v>
-      </c>
-    </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="B33" s="20">
+      <c r="A33" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B35" s="17"/>
+      <c r="D35" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="E35" s="17"/>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="B36" s="23">
         <f>B10</f>
         <v>0</v>
       </c>
-      <c r="D33" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="E33" s="20">
-        <f>B17</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
+      <c r="D36" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E36" s="23">
+        <f>B19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="B37" s="21">
+        <f>'Monthly Bills'!B23</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" s="21">
+        <f>'Monthly Bills'!B24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="B38" s="23">
+        <f>B12</f>
+        <v>0</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="E38" s="23">
+        <f>B21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="B39" s="23">
+        <f>C13</f>
+        <v>0</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="E39" s="23">
+        <f>C22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B40" s="23">
+        <f>D13</f>
+        <v>0</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="E40" s="23">
+        <f>D22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="B41" s="23">
+        <f>E13</f>
+        <v>0</v>
+      </c>
+      <c r="D41" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="E41" s="23">
+        <f>E22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="B43" s="25"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="25"/>
+      <c r="E43" s="25"/>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="B44" s="26"/>
+      <c r="C44" s="26"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="26"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A44:E44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2908,7 +3158,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2917,7 +3167,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2926,7 +3176,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -2938,7 +3188,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -2953,23 +3203,23 @@
         <v>0</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E6" s="8">
-        <f>'Monthly Bills'!B67+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B76+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="7" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="B7" s="8">
         <f>'Monthly Bills'!B7</f>
         <v>0</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="E7" s="8">
         <f>'Monthly Bills'!B19</f>
@@ -2978,56 +3228,63 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="B8" s="10">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="E8" s="8">
-        <f>'Monthly Bills'!B8-E6-E7</f>
+        <f>'Monthly Bills'!B8-E6-E7-'Monthly Bills'!B25-'Monthly Bills'!B26</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="D9" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="E9" s="10">
-        <f>SUM(E6:E8)</f>
+      <c r="D9" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E9" s="8">
+        <f>'Monthly Bills'!B25+'Monthly Bills'!B26</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="B10" s="3"/>
+      <c r="D10" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="E10" s="10">
+        <f>SUM(E6:E9)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="B11" s="23">
+        <v>90</v>
+      </c>
+      <c r="B11" s="27">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="B12" s="24">
-        <f>'Monthly Bills'!B67</f>
+        <v>116</v>
+      </c>
+      <c r="B12" s="28">
+        <f>'Monthly Bills'!B74</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="7" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B13" s="8">
         <f>'Monthly Bills'!B18</f>
@@ -3036,7 +3293,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="7" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="B14" s="8">
         <f>'Monthly Bills'!B19</f>
@@ -3045,20 +3302,20 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="B15" s="23">
+        <v>119</v>
+      </c>
+      <c r="B15" s="27">
         <f>E8</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="11" t="s">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="B17" s="11"/>
       <c r="D17" s="11" t="s">
-        <v>104</v>
+        <v>121</v>
       </c>
       <c r="E17" s="11"/>
     </row>
@@ -3070,7 +3327,7 @@
         <v>4</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>4</v>
@@ -3085,10 +3342,10 @@
         <v>0</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="E19" s="13">
-        <f>'Monthly Bills'!B67+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B76+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
     </row>
@@ -3101,7 +3358,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="E20" s="13">
         <f>'Monthly Bills'!B19</f>
@@ -3117,31 +3374,38 @@
         <v>0</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="E21" s="13">
-        <f>'Monthly Bills'!B14-E19-E20</f>
+        <f>'Monthly Bills'!B14-E19-E20-'Monthly Bills'!B25-'Monthly Bills'!B26</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="D22" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="E22" s="15">
-        <f>SUM(E19:E21)</f>
+      <c r="D22" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="E22" s="13">
+        <f>'Monthly Bills'!B25+'Monthly Bills'!B26</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="11" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="B23" s="11"/>
+      <c r="D23" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" s="15">
+        <f>SUM(E19:E22)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="12" t="s">
-        <v>106</v>
+        <v>123</v>
       </c>
       <c r="B24" s="13">
         <f>'Monthly Bills'!B14</f>
@@ -3150,16 +3414,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="12" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="B25" s="13">
-        <f>'Monthly Bills'!B67</f>
+        <f>'Monthly Bills'!B74</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="12" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B26" s="13">
         <f>'Monthly Bills'!B18</f>
@@ -3168,7 +3432,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="12" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="B27" s="13">
         <f>'Monthly Bills'!B19</f>
@@ -3177,7 +3441,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="12" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="B28" s="13">
         <f>E21</f>
@@ -3186,7 +3450,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="14" t="s">
-        <v>108</v>
+        <v>125</v>
       </c>
       <c r="B29" s="15">
         <f>B28-B15</f>
@@ -3222,7 +3486,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3233,26 +3497,26 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" s="11" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" s="23">
+        <v>128</v>
+      </c>
+      <c r="B4" s="27">
         <f>Overview!E8</f>
         <v>0</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="F4" s="13">
         <f>Overview!E21</f>
@@ -3261,219 +3525,219 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="B7" s="6">
         <v>350</v>
       </c>
-      <c r="C7" s="25">
+      <c r="C7" s="29">
         <f>IF($B$4&gt;0,B7/$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="F7" s="13">
         <f>B7</f>
         <v>0</v>
       </c>
-      <c r="G7" s="26">
+      <c r="G7" s="30">
         <f>IF($F$4&gt;0,F7/$F$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="5" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="B8" s="6">
         <v>225</v>
       </c>
-      <c r="C8" s="25">
+      <c r="C8" s="29">
         <f>IF($B$4&gt;0,B8/$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="F8" s="13">
         <f>B8</f>
         <v>0</v>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="30">
         <f>IF($F$4&gt;0,F8/$F$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="B9" s="6">
         <v>225</v>
       </c>
-      <c r="C9" s="25">
+      <c r="C9" s="29">
         <f>IF($B$4&gt;0,B9/$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="F9" s="13">
         <f>B9</f>
         <v>0</v>
       </c>
-      <c r="G9" s="26">
+      <c r="G9" s="30">
         <f>IF($F$4&gt;0,F9/$F$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="5" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="B10" s="6">
         <v>175</v>
       </c>
-      <c r="C10" s="25">
+      <c r="C10" s="29">
         <f>IF($B$4&gt;0,B10/$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="F10" s="13">
         <f>B10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="26">
+      <c r="G10" s="30">
         <f>IF($F$4&gt;0,F10/$F$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="B11" s="6">
         <v>150</v>
       </c>
-      <c r="C11" s="25">
+      <c r="C11" s="29">
         <f>IF($B$4&gt;0,B11/$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="F11" s="13">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="26">
+      <c r="G11" s="30">
         <f>IF($F$4&gt;0,F11/$F$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="B12" s="6">
         <v>150</v>
       </c>
-      <c r="C12" s="25">
+      <c r="C12" s="29">
         <f>IF($B$4&gt;0,B12/$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="F12" s="13">
         <f>B12</f>
         <v>0</v>
       </c>
-      <c r="G12" s="26">
+      <c r="G12" s="30">
         <f>IF($F$4&gt;0,F12/$F$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="5" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="B13" s="6">
         <v>100</v>
       </c>
-      <c r="C13" s="25">
+      <c r="C13" s="29">
         <f>IF($B$4&gt;0,B13/$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="F13" s="13">
         <f>B13</f>
         <v>0</v>
       </c>
-      <c r="G13" s="26">
+      <c r="G13" s="30">
         <f>IF($F$4&gt;0,F13/$F$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="B14" s="10">
         <f>$B$4-SUM(B7:B13)</f>
         <v>0</v>
       </c>
-      <c r="C14" s="27">
+      <c r="C14" s="31">
         <f>IF($B$4&gt;0,B14/$B$4,0)</f>
         <v>0</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="F14" s="15">
         <f>$F$4-SUM(F7:F13)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="28">
+      <c r="G14" s="32">
         <f>IF($F$4&gt;0,F14/$F$4,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="B16" s="10">
         <f>SUM(B7:B14)</f>
         <v>0</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="F16" s="15">
         <f>SUM(F7:F14)</f>
@@ -3482,7 +3746,7 @@
     </row>
     <row r="18" spans="5:6">
       <c r="E18" s="14" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="F18" s="15">
         <f>F14-B14</f>

</xml_diff>

<commit_message>
Add subscriptions: Apple iCloud (.99), Apple Music (cd /workspace && python3 create_budget.py && git add Family_Budget.xlsx && git commit -m "Add subscriptions: Apple iCloud ($9.99), Apple Music ($19.99), Apple iCloud 2 ($0.99), Netflix ($28.88)" && git push9.99), Apple iCloud 2 (--.99), Netflix (8.88)
Co-authored-by: jbox662 <jbox662@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Family_Budget.xlsx
+++ b/Family_Budget.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="150">
   <si>
     <t>MONTHLY BILLS - EDIT HERE</t>
   </si>
@@ -175,6 +175,24 @@
     <t>Debt Total</t>
   </si>
   <si>
+    <t>SUBSCRIPTIONS</t>
+  </si>
+  <si>
+    <t>Apple iCloud</t>
+  </si>
+  <si>
+    <t>Apple Music</t>
+  </si>
+  <si>
+    <t>Apple iCloud (2nd)</t>
+  </si>
+  <si>
+    <t>Netflix</t>
+  </si>
+  <si>
+    <t>Subscriptions Total</t>
+  </si>
+  <si>
     <t>OTHER EXPENSES</t>
   </si>
   <si>
@@ -221,6 +239,9 @@
   </si>
   <si>
     <t>Debt Payments</t>
+  </si>
+  <si>
+    <t>Subscriptions</t>
   </si>
   <si>
     <t>Other</t>
@@ -829,9 +850,9 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>'Monthly Bills'!$D$6:$D$11</c:f>
+              <c:f>'Monthly Bills'!$D$6:$D$12</c:f>
               <c:strCache>
-                <c:ptCount val="6"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Vehicles</c:v>
                 </c:pt>
@@ -848,6 +869,9 @@
                   <c:v>Debt Payments</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>Subscriptions</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>Other</c:v>
                 </c:pt>
               </c:strCache>
@@ -855,10 +879,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Monthly Bills'!$E$6:$E$11</c:f>
+              <c:f>'Monthly Bills'!$E$6:$E$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -875,6 +899,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -999,9 +1026,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Monthly Bills'!$D$6:$D$11</c:f>
+              <c:f>'Monthly Bills'!$D$6:$D$12</c:f>
               <c:strCache>
-                <c:ptCount val="6"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Vehicles</c:v>
                 </c:pt>
@@ -1018,6 +1045,9 @@
                   <c:v>Debt Payments</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>Subscriptions</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>Other</c:v>
                 </c:pt>
               </c:strCache>
@@ -1025,10 +1055,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Monthly Bills'!$E$6:$E$11</c:f>
+              <c:f>'Monthly Bills'!$E$6:$E$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1045,6 +1075,9 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -2030,7 +2063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -2057,7 +2090,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -2069,7 +2102,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -2083,7 +2116,7 @@
         <v>6000</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E6" s="8">
         <f>B34</f>
@@ -2098,7 +2131,7 @@
         <v>4875.5</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E7" s="8">
         <f>B41</f>
@@ -2114,7 +2147,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="E8" s="8">
         <f>B50</f>
@@ -2123,7 +2156,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="7" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E9" s="8">
         <f>B56</f>
@@ -2136,7 +2169,7 @@
       </c>
       <c r="B10" s="11"/>
       <c r="D10" s="7" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E10" s="8">
         <f>B64</f>
@@ -2151,10 +2184,10 @@
         <v>4</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="E11" s="8">
-        <f>B71</f>
+        <f>B72</f>
         <v>0</v>
       </c>
     </row>
@@ -2166,6 +2199,13 @@
         <f>B6</f>
         <v>0</v>
       </c>
+      <c r="D12" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" s="8">
+        <f>B79</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="12" t="s">
@@ -2541,7 +2581,7 @@
         <v>53</v>
       </c>
       <c r="B68" s="6">
-        <v>600</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -2549,7 +2589,7 @@
         <v>54</v>
       </c>
       <c r="B69" s="6">
-        <v>100</v>
+        <v>19.99</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -2557,53 +2597,108 @@
         <v>55</v>
       </c>
       <c r="B70" s="6">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B71" s="6">
+        <v>28.88</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B72" s="10">
+        <f>SUM(B68:B71)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B74" s="3"/>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B76" s="6">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B77" s="6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B78" s="6">
         <v>240</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
-      <c r="A71" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B71" s="10">
-        <f>SUM(B68:B70)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2">
-      <c r="A73" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B73" s="3"/>
-    </row>
-    <row r="74" spans="1:2">
-      <c r="A74" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B74" s="10">
-        <f>B34+B41+B50+B56+B64+B71</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2">
-      <c r="A75" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B75" s="8">
+    <row r="79" spans="1:2">
+      <c r="A79" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B79" s="10">
+        <f>SUM(B76:B78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B81" s="3"/>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B82" s="10">
+        <f>B34+B41+B50+B56+B64+B72+B79</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B83" s="8">
         <f>B25+B26</f>
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
-      <c r="A76" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="B76" s="10">
-        <f>B74-B75</f>
+    <row r="84" spans="1:2">
+      <c r="A84" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B84" s="10">
+        <f>B82-B83</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A10:B10"/>
@@ -2615,7 +2710,8 @@
     <mergeCell ref="A52:B52"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A81:B81"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2634,7 +2730,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2643,12 +2739,12 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -2658,28 +2754,28 @@
     <row r="5" spans="1:5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B6" s="10">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
       <c r="C6" s="10">
-        <f>'Monthly Bills'!B76+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B84+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
       <c r="D6" s="10">
@@ -2693,7 +2789,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="17" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -2706,18 +2802,18 @@
         <v>4</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="18" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B10" s="19">
         <f>'Monthly Bills'!B6/2</f>
@@ -2726,7 +2822,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="20" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B11" s="21">
         <f>-'Monthly Bills'!B23</f>
@@ -2735,7 +2831,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="22" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B12" s="23">
         <f>B10+B11</f>
@@ -2744,7 +2840,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="18" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B13" s="19">
         <f>B12</f>
@@ -2765,7 +2861,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="22" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B14" s="23">
         <f>B13*2</f>
@@ -2786,7 +2882,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="20" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B15" s="21">
         <f>'Monthly Bills'!B25</f>
@@ -2795,7 +2891,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="17" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -2808,18 +2904,18 @@
         <v>4</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="18" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B19" s="19">
         <f>'Monthly Bills'!B7/2.167</f>
@@ -2828,7 +2924,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="20" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B20" s="21">
         <f>-'Monthly Bills'!B24</f>
@@ -2837,7 +2933,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="22" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B21" s="23">
         <f>B19+B20</f>
@@ -2846,7 +2942,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="18" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B22" s="19">
         <f>B21</f>
@@ -2867,7 +2963,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="22" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B23" s="23">
         <f>B22*2.167</f>
@@ -2888,7 +2984,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="20" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B24" s="21">
         <f>'Monthly Bills'!B26</f>
@@ -2897,7 +2993,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -2907,21 +3003,21 @@
     <row r="27" spans="1:5">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="9" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B28" s="10">
         <f>B14+B23</f>
@@ -2942,19 +3038,19 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="20" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B29" s="21">
         <f>B15+B24</f>
         <v>0</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="22" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="B30" s="23">
         <f>B28+B29</f>
@@ -2975,7 +3071,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="7" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B31" s="8">
         <f>B6</f>
@@ -2996,7 +3092,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="24" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B33" s="24"/>
       <c r="C33" s="24"/>
@@ -3005,24 +3101,24 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="17" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B35" s="17"/>
       <c r="D35" s="17" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="E35" s="17"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="18" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B36" s="23">
         <f>B10</f>
         <v>0</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E36" s="23">
         <f>B19</f>
@@ -3031,14 +3127,14 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="20" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B37" s="21">
         <f>'Monthly Bills'!B23</f>
         <v>0</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="E37" s="21">
         <f>'Monthly Bills'!B24</f>
@@ -3047,14 +3143,14 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="22" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B38" s="23">
         <f>B12</f>
         <v>0</v>
       </c>
       <c r="D38" s="22" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="E38" s="23">
         <f>B21</f>
@@ -3063,14 +3159,14 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="18" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B39" s="23">
         <f>C13</f>
         <v>0</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="E39" s="23">
         <f>C22</f>
@@ -3079,14 +3175,14 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="18" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="B40" s="23">
         <f>D13</f>
         <v>0</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="E40" s="23">
         <f>D22</f>
@@ -3095,14 +3191,14 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="18" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B41" s="23">
         <f>E13</f>
         <v>0</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E41" s="23">
         <f>E22</f>
@@ -3111,7 +3207,7 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="25" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B43" s="25"/>
       <c r="C43" s="25"/>
@@ -3120,7 +3216,7 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="26" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B44" s="26"/>
       <c r="C44" s="26"/>
@@ -3158,7 +3254,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3167,7 +3263,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3176,7 +3272,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -3188,7 +3284,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -3203,23 +3299,23 @@
         <v>0</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E6" s="8">
-        <f>'Monthly Bills'!B76+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B84+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="7" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B7" s="8">
         <f>'Monthly Bills'!B7</f>
         <v>0</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E7" s="8">
         <f>'Monthly Bills'!B19</f>
@@ -3228,14 +3324,14 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B8" s="10">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E8" s="8">
         <f>'Monthly Bills'!B8-E6-E7-'Monthly Bills'!B25-'Monthly Bills'!B26</f>
@@ -3244,7 +3340,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="7" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E9" s="8">
         <f>'Monthly Bills'!B25+'Monthly Bills'!B26</f>
@@ -3253,11 +3349,11 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B10" s="3"/>
       <c r="D10" s="9" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="E10" s="10">
         <f>SUM(E6:E9)</f>
@@ -3266,7 +3362,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="B11" s="27">
         <f>'Monthly Bills'!B8</f>
@@ -3275,16 +3371,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B12" s="28">
-        <f>'Monthly Bills'!B74</f>
+        <f>'Monthly Bills'!B82</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="7" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B13" s="8">
         <f>'Monthly Bills'!B18</f>
@@ -3293,7 +3389,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="7" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B14" s="8">
         <f>'Monthly Bills'!B19</f>
@@ -3302,7 +3398,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="7" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B15" s="27">
         <f>E8</f>
@@ -3311,11 +3407,11 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="11" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B17" s="11"/>
       <c r="D17" s="11" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="E17" s="11"/>
     </row>
@@ -3327,7 +3423,7 @@
         <v>4</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>4</v>
@@ -3342,10 +3438,10 @@
         <v>0</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E19" s="13">
-        <f>'Monthly Bills'!B76+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B84+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
     </row>
@@ -3358,7 +3454,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="E20" s="13">
         <f>'Monthly Bills'!B19</f>
@@ -3374,7 +3470,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E21" s="13">
         <f>'Monthly Bills'!B14-E19-E20-'Monthly Bills'!B25-'Monthly Bills'!B26</f>
@@ -3383,7 +3479,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="D22" s="12" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="E22" s="13">
         <f>'Monthly Bills'!B25+'Monthly Bills'!B26</f>
@@ -3392,11 +3488,11 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="11" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B23" s="11"/>
       <c r="D23" s="14" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="E23" s="15">
         <f>SUM(E19:E22)</f>
@@ -3405,7 +3501,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="12" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B24" s="13">
         <f>'Monthly Bills'!B14</f>
@@ -3414,16 +3510,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="12" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B25" s="13">
-        <f>'Monthly Bills'!B74</f>
+        <f>'Monthly Bills'!B82</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="12" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B26" s="13">
         <f>'Monthly Bills'!B18</f>
@@ -3432,7 +3528,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="12" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B27" s="13">
         <f>'Monthly Bills'!B19</f>
@@ -3441,7 +3537,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="12" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B28" s="13">
         <f>E21</f>
@@ -3450,7 +3546,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="14" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B29" s="15">
         <f>B28-B15</f>
@@ -3486,7 +3582,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3497,26 +3593,26 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" s="11" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="7" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B4" s="27">
         <f>Overview!E8</f>
         <v>0</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="F4" s="13">
         <f>Overview!E21</f>
@@ -3525,27 +3621,27 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B7" s="6">
         <v>350</v>
@@ -3555,7 +3651,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="F7" s="13">
         <f>B7</f>
@@ -3568,7 +3664,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="5" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B8" s="6">
         <v>225</v>
@@ -3578,7 +3674,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="F8" s="13">
         <f>B8</f>
@@ -3591,7 +3687,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B9" s="6">
         <v>225</v>
@@ -3601,7 +3697,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="F9" s="13">
         <f>B9</f>
@@ -3614,7 +3710,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="5" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="B10" s="6">
         <v>175</v>
@@ -3624,7 +3720,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="F10" s="13">
         <f>B10</f>
@@ -3637,7 +3733,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="B11" s="6">
         <v>150</v>
@@ -3647,7 +3743,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F11" s="13">
         <f>B11</f>
@@ -3660,7 +3756,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B12" s="6">
         <v>150</v>
@@ -3670,7 +3766,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="F12" s="13">
         <f>B12</f>
@@ -3683,7 +3779,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="5" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B13" s="6">
         <v>100</v>
@@ -3693,7 +3789,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="F13" s="13">
         <f>B13</f>
@@ -3706,7 +3802,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B14" s="10">
         <f>$B$4-SUM(B7:B13)</f>
@@ -3717,7 +3813,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="F14" s="15">
         <f>$F$4-SUM(F7:F13)</f>
@@ -3730,14 +3826,14 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B16" s="10">
         <f>SUM(B7:B14)</f>
         <v>0</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="F16" s="15">
         <f>SUM(F7:F14)</f>
@@ -3746,7 +3842,7 @@
     </row>
     <row r="18" spans="5:6">
       <c r="E18" s="14" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="F18" s="15">
         <f>F14-B14</f>

</xml_diff>

<commit_message>
Add Business Insurance (5.33)
Co-authored-by: jbox662 <jbox662@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Family_Budget.xlsx
+++ b/Family_Budget.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="151">
   <si>
     <t>MONTHLY BILLS - EDIT HERE</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>Man Life</t>
+  </si>
+  <si>
+    <t>Business Insurance</t>
   </si>
   <si>
     <t>Insurance Total</t>
@@ -2063,7 +2066,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -2090,7 +2093,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -2102,7 +2105,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -2116,7 +2119,7 @@
         <v>6000</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E6" s="8">
         <f>B34</f>
@@ -2131,7 +2134,7 @@
         <v>4875.5</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E7" s="8">
         <f>B41</f>
@@ -2147,7 +2150,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E8" s="8">
         <f>B50</f>
@@ -2156,10 +2159,10 @@
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E9" s="8">
-        <f>B56</f>
+        <f>B57</f>
         <v>0</v>
       </c>
     </row>
@@ -2169,10 +2172,10 @@
       </c>
       <c r="B10" s="11"/>
       <c r="D10" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E10" s="8">
-        <f>B64</f>
+        <f>B65</f>
         <v>0</v>
       </c>
     </row>
@@ -2184,10 +2187,10 @@
         <v>4</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E11" s="8">
-        <f>B72</f>
+        <f>B73</f>
         <v>0</v>
       </c>
     </row>
@@ -2200,10 +2203,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E12" s="8">
-        <f>B79</f>
+        <f>B80</f>
         <v>0</v>
       </c>
     </row>
@@ -2499,34 +2502,34 @@
       </c>
     </row>
     <row r="56" spans="1:2">
-      <c r="A56" s="9" t="s">
+      <c r="A56" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B56" s="10">
-        <f>SUM(B54:B55)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" s="3" t="s">
+      <c r="B56" s="6">
+        <v>45.33</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B58" s="3"/>
+      <c r="B57" s="10">
+        <f>SUM(B54:B56)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="59" spans="1:2">
-      <c r="A59" s="4" t="s">
+      <c r="A59" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B59" s="3"/>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B60" s="4" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2">
-      <c r="A60" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B60" s="6">
-        <v>105</v>
       </c>
     </row>
     <row r="61" spans="1:2">
@@ -2534,7 +2537,7 @@
         <v>48</v>
       </c>
       <c r="B61" s="6">
-        <v>106.16</v>
+        <v>105</v>
       </c>
     </row>
     <row r="62" spans="1:2">
@@ -2542,7 +2545,7 @@
         <v>49</v>
       </c>
       <c r="B62" s="6">
-        <v>338</v>
+        <v>106.16</v>
       </c>
     </row>
     <row r="63" spans="1:2">
@@ -2550,38 +2553,38 @@
         <v>50</v>
       </c>
       <c r="B63" s="6">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B64" s="6">
         <v>519</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
-      <c r="A64" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B64" s="10">
-        <f>SUM(B60:B63)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2">
-      <c r="A66" s="3" t="s">
+    <row r="65" spans="1:2">
+      <c r="A65" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B66" s="3"/>
+      <c r="B65" s="10">
+        <f>SUM(B61:B64)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="67" spans="1:2">
-      <c r="A67" s="4" t="s">
+      <c r="A67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B67" s="3"/>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B68" s="4" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2">
-      <c r="A68" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B68" s="6">
-        <v>9.99</v>
       </c>
     </row>
     <row r="69" spans="1:2">
@@ -2589,7 +2592,7 @@
         <v>54</v>
       </c>
       <c r="B69" s="6">
-        <v>19.99</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="70" spans="1:2">
@@ -2597,7 +2600,7 @@
         <v>55</v>
       </c>
       <c r="B70" s="6">
-        <v>0.99</v>
+        <v>19.99</v>
       </c>
     </row>
     <row r="71" spans="1:2">
@@ -2605,38 +2608,38 @@
         <v>56</v>
       </c>
       <c r="B71" s="6">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B72" s="6">
         <v>28.88</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
-      <c r="A72" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="B72" s="10">
-        <f>SUM(B68:B71)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2">
-      <c r="A74" s="3" t="s">
+    <row r="73" spans="1:2">
+      <c r="A73" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B74" s="3"/>
+      <c r="B73" s="10">
+        <f>SUM(B69:B72)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="75" spans="1:2">
-      <c r="A75" s="4" t="s">
+      <c r="A75" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B75" s="3"/>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B75" s="4" t="s">
+      <c r="B76" s="4" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2">
-      <c r="A76" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B76" s="6">
-        <v>600</v>
       </c>
     </row>
     <row r="77" spans="1:2">
@@ -2644,7 +2647,7 @@
         <v>60</v>
       </c>
       <c r="B77" s="6">
-        <v>100</v>
+        <v>600</v>
       </c>
     </row>
     <row r="78" spans="1:2">
@@ -2652,48 +2655,56 @@
         <v>61</v>
       </c>
       <c r="B78" s="6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B79" s="6">
         <v>240</v>
       </c>
     </row>
-    <row r="79" spans="1:2">
-      <c r="A79" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="B79" s="10">
-        <f>SUM(B76:B78)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2">
-      <c r="A81" s="3" t="s">
+    <row r="80" spans="1:2">
+      <c r="A80" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B81" s="3"/>
+      <c r="B80" s="10">
+        <f>SUM(B77:B79)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="82" spans="1:2">
-      <c r="A82" s="9" t="s">
+      <c r="A82" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B82" s="10">
-        <f>B34+B41+B50+B56+B64+B72+B79</f>
-        <v>0</v>
-      </c>
+      <c r="B82" s="3"/>
     </row>
     <row r="83" spans="1:2">
-      <c r="A83" s="7" t="s">
+      <c r="A83" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B83" s="8">
+      <c r="B83" s="10">
+        <f>B34+B41+B50+B57+B65+B73+B80</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="B84" s="8">
         <f>B25+B26</f>
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
-      <c r="A84" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="B84" s="10">
-        <f>B82-B83</f>
+    <row r="85" spans="1:2">
+      <c r="A85" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B85" s="10">
+        <f>B83-B84</f>
         <v>0</v>
       </c>
     </row>
@@ -2708,10 +2719,10 @@
     <mergeCell ref="A36:B36"/>
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="A82:B82"/>
     <mergeCell ref="D4:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2730,7 +2741,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2739,12 +2750,12 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -2754,28 +2765,28 @@
     <row r="5" spans="1:5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B6" s="10">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
       <c r="C6" s="10">
-        <f>'Monthly Bills'!B84+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B85+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
       <c r="D6" s="10">
@@ -2789,7 +2800,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="17" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -2802,18 +2813,18 @@
         <v>4</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B10" s="19">
         <f>'Monthly Bills'!B6/2</f>
@@ -2822,7 +2833,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B11" s="21">
         <f>-'Monthly Bills'!B23</f>
@@ -2831,7 +2842,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B12" s="23">
         <f>B10+B11</f>
@@ -2840,7 +2851,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B13" s="19">
         <f>B12</f>
@@ -2861,7 +2872,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="22" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B14" s="23">
         <f>B13*2</f>
@@ -2882,7 +2893,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" s="21">
         <f>'Monthly Bills'!B25</f>
@@ -2891,7 +2902,7 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -2904,18 +2915,18 @@
         <v>4</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B19" s="19">
         <f>'Monthly Bills'!B7/2.167</f>
@@ -2924,7 +2935,7 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="20" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B20" s="21">
         <f>-'Monthly Bills'!B24</f>
@@ -2933,7 +2944,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="22" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B21" s="23">
         <f>B19+B20</f>
@@ -2942,7 +2953,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B22" s="19">
         <f>B21</f>
@@ -2963,7 +2974,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="22" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B23" s="23">
         <f>B22*2.167</f>
@@ -2984,7 +2995,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B24" s="21">
         <f>'Monthly Bills'!B26</f>
@@ -2993,7 +3004,7 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -3003,21 +3014,21 @@
     <row r="27" spans="1:5">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B28" s="10">
         <f>B14+B23</f>
@@ -3038,19 +3049,19 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B29" s="21">
         <f>B15+B24</f>
         <v>0</v>
       </c>
       <c r="C29" s="20" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="22" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B30" s="23">
         <f>B28+B29</f>
@@ -3071,7 +3082,7 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B31" s="8">
         <f>B6</f>
@@ -3092,7 +3103,7 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B33" s="24"/>
       <c r="C33" s="24"/>
@@ -3101,24 +3112,24 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B35" s="17"/>
       <c r="D35" s="17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E35" s="17"/>
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B36" s="23">
         <f>B10</f>
         <v>0</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E36" s="23">
         <f>B19</f>
@@ -3127,14 +3138,14 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B37" s="21">
         <f>'Monthly Bills'!B23</f>
         <v>0</v>
       </c>
       <c r="D37" s="20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E37" s="21">
         <f>'Monthly Bills'!B24</f>
@@ -3143,14 +3154,14 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B38" s="23">
         <f>B12</f>
         <v>0</v>
       </c>
       <c r="D38" s="22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E38" s="23">
         <f>B21</f>
@@ -3159,14 +3170,14 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B39" s="23">
         <f>C13</f>
         <v>0</v>
       </c>
       <c r="D39" s="18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E39" s="23">
         <f>C22</f>
@@ -3175,14 +3186,14 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B40" s="23">
         <f>D13</f>
         <v>0</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E40" s="23">
         <f>D22</f>
@@ -3191,14 +3202,14 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B41" s="23">
         <f>E13</f>
         <v>0</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E41" s="23">
         <f>E22</f>
@@ -3207,7 +3218,7 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="25" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B43" s="25"/>
       <c r="C43" s="25"/>
@@ -3216,7 +3227,7 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B44" s="26"/>
       <c r="C44" s="26"/>
@@ -3254,7 +3265,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3263,7 +3274,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3272,7 +3283,7 @@
       </c>
       <c r="B4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E4" s="3"/>
     </row>
@@ -3284,7 +3295,7 @@
         <v>4</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>4</v>
@@ -3299,23 +3310,23 @@
         <v>0</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E6" s="8">
-        <f>'Monthly Bills'!B84+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B85+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B7" s="8">
         <f>'Monthly Bills'!B7</f>
         <v>0</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E7" s="8">
         <f>'Monthly Bills'!B19</f>
@@ -3324,14 +3335,14 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B8" s="10">
         <f>'Monthly Bills'!B8</f>
         <v>0</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E8" s="8">
         <f>'Monthly Bills'!B8-E6-E7-'Monthly Bills'!B25-'Monthly Bills'!B26</f>
@@ -3340,7 +3351,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="D9" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E9" s="8">
         <f>'Monthly Bills'!B25+'Monthly Bills'!B26</f>
@@ -3349,11 +3360,11 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B10" s="3"/>
       <c r="D10" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E10" s="10">
         <f>SUM(E6:E9)</f>
@@ -3362,7 +3373,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B11" s="27">
         <f>'Monthly Bills'!B8</f>
@@ -3371,16 +3382,16 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B12" s="28">
-        <f>'Monthly Bills'!B82</f>
+        <f>'Monthly Bills'!B83</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B13" s="8">
         <f>'Monthly Bills'!B18</f>
@@ -3389,7 +3400,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B14" s="8">
         <f>'Monthly Bills'!B19</f>
@@ -3398,7 +3409,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B15" s="27">
         <f>E8</f>
@@ -3407,11 +3418,11 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B17" s="11"/>
       <c r="D17" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E17" s="11"/>
     </row>
@@ -3423,7 +3434,7 @@
         <v>4</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>4</v>
@@ -3438,10 +3449,10 @@
         <v>0</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E19" s="13">
-        <f>'Monthly Bills'!B84+'Monthly Bills'!B18</f>
+        <f>'Monthly Bills'!B85+'Monthly Bills'!B18</f>
         <v>0</v>
       </c>
     </row>
@@ -3454,7 +3465,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E20" s="13">
         <f>'Monthly Bills'!B19</f>
@@ -3470,7 +3481,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E21" s="13">
         <f>'Monthly Bills'!B14-E19-E20-'Monthly Bills'!B25-'Monthly Bills'!B26</f>
@@ -3479,7 +3490,7 @@
     </row>
     <row r="22" spans="1:5">
       <c r="D22" s="12" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E22" s="13">
         <f>'Monthly Bills'!B25+'Monthly Bills'!B26</f>
@@ -3488,11 +3499,11 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="11" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B23" s="11"/>
       <c r="D23" s="14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E23" s="15">
         <f>SUM(E19:E22)</f>
@@ -3501,7 +3512,7 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B24" s="13">
         <f>'Monthly Bills'!B14</f>
@@ -3510,16 +3521,16 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B25" s="13">
-        <f>'Monthly Bills'!B82</f>
+        <f>'Monthly Bills'!B83</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B26" s="13">
         <f>'Monthly Bills'!B18</f>
@@ -3528,7 +3539,7 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B27" s="13">
         <f>'Monthly Bills'!B19</f>
@@ -3537,7 +3548,7 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="12" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B28" s="13">
         <f>E21</f>
@@ -3546,7 +3557,7 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="14" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B29" s="15">
         <f>B28-B15</f>
@@ -3582,7 +3593,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3593,26 +3604,26 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B4" s="27">
         <f>Overview!E8</f>
         <v>0</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F4" s="13">
         <f>Overview!E21</f>
@@ -3621,27 +3632,27 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>136</v>
-      </c>
       <c r="G6" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B7" s="6">
         <v>350</v>
@@ -3651,7 +3662,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F7" s="13">
         <f>B7</f>
@@ -3664,7 +3675,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B8" s="6">
         <v>225</v>
@@ -3674,7 +3685,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F8" s="13">
         <f>B8</f>
@@ -3687,7 +3698,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B9" s="6">
         <v>225</v>
@@ -3697,7 +3708,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F9" s="13">
         <f>B9</f>
@@ -3710,7 +3721,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B10" s="6">
         <v>175</v>
@@ -3720,7 +3731,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F10" s="13">
         <f>B10</f>
@@ -3733,7 +3744,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B11" s="6">
         <v>150</v>
@@ -3743,7 +3754,7 @@
         <v>0</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F11" s="13">
         <f>B11</f>
@@ -3756,7 +3767,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B12" s="6">
         <v>150</v>
@@ -3766,7 +3777,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F12" s="13">
         <f>B12</f>
@@ -3779,7 +3790,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B13" s="6">
         <v>100</v>
@@ -3789,7 +3800,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F13" s="13">
         <f>B13</f>
@@ -3802,7 +3813,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B14" s="10">
         <f>$B$4-SUM(B7:B13)</f>
@@ -3813,7 +3824,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F14" s="15">
         <f>$F$4-SUM(F7:F13)</f>
@@ -3826,14 +3837,14 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B16" s="10">
         <f>SUM(B7:B14)</f>
         <v>0</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F16" s="15">
         <f>SUM(F7:F14)</f>
@@ -3842,7 +3853,7 @@
     </row>
     <row r="18" spans="5:6">
       <c r="E18" s="14" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F18" s="15">
         <f>F14-B14</f>

</xml_diff>

<commit_message>
Fix spending formulas - you put more in spending since you have higher take-home after DD
Co-authored-by: jbox662 <jbox662@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Family_Budget.xlsx
+++ b/Family_Budget.xlsx
@@ -2866,7 +2866,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="19">
-        <f>B13-C13-D13</f>
+        <f>B12-C13-D13</f>
         <v>0</v>
       </c>
     </row>
@@ -2968,7 +2968,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="19">
-        <f>B22-C22-D22</f>
+        <f>B21-C22-D22</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>